<commit_message>
Complete Xcode simulator readiness setup
</commit_message>
<xml_diff>
--- a/ios-app-readiness/iOS_App_Readiness_Tracker.xlsx
+++ b/ios-app-readiness/iOS_App_Readiness_Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0523b0d89d7a4f09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="2" r:id="Ra04750d52f464bdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checklist" sheetId="3" r:id="R3aa998247d4147d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Map" sheetId="4" r:id="Rb625619fdc834bbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R9b89c3d4343d4f90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9fb08bbe167643ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="2" r:id="Rf8180201b7964135"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checklist" sheetId="3" r:id="Rab250d69b01c4e0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Map" sheetId="4" r:id="R46bdab8948e14616"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R12f1321f28574a3f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -507,7 +507,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -1276,7 +1276,7 @@
       </x:c>
       <x:c r="B27" s="27" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"In Progress")</x:f>
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
@@ -1294,7 +1294,7 @@
       </x:c>
       <x:c r="B29" s="27" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"Not Started")</x:f>
-        <x:v>21</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1712,10 +1712,10 @@
         <x:v>APPLE-SUBMIT</x:v>
       </x:c>
       <x:c r="K13" s="21" t="str">
-        <x:v>Capacitor 8 Xcode project created with the approved bundle ID. Full Xcode/iOS SDK, signing, simulator, and device launch remain prerequisites.</x:v>
+        <x:v>Capacitor 8 Xcode project created with approved bundle ID. Xcode 26.6 selected; first launch complete; iOS 26.5 simulator mounted; Swift packages resolved; unsigned Debug builds launch on iPhone 17 Pro/iPad Pro 13-inch. Signing/Developer enrollment remain.</x:v>
       </x:c>
       <x:c r="L13" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46266</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -1864,10 +1864,10 @@
         <x:v>PROJECT</x:v>
       </x:c>
       <x:c r="K17" s="21" t="str">
-        <x:v>Pinned 146 MB runtime/package closure built and browser-smoke tested locally. Clean-install/offline recovery still needs iOS devices.</x:v>
+        <x:v>Pinned 146 MB runtime/package closure built and browser-smoke tested. npm ci, npm run ios:sync, and npm run check pass. Clean-install simulator launch reached home; offline/runtime recovery still needs validation.</x:v>
       </x:c>
       <x:c r="L17" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46266</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
@@ -1976,10 +1976,10 @@
         <x:v>APPLE-QA</x:v>
       </x:c>
       <x:c r="K20" s="21" t="str">
-        <x:v>Requires physical-device testing, not only desktop browser testing.</x:v>
+        <x:v>Simulator build/launch smoke passes, but WebKit feature coverage and physical-device testing remain.</x:v>
       </x:c>
       <x:c r="L20" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46266</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
@@ -2204,10 +2204,10 @@
         <x:v>APPLE-ICON</x:v>
       </x:c>
       <x:c r="K26" s="21" t="str">
-        <x:v>Final-direction icon, branded launch assets, status-bar configuration, and safe-area styling are installed. Home Screen/TestFlight review remains.</x:v>
+        <x:v>Final-direction icon, branded launch assets, status-bar configuration, and safe-area styling are installed. Simulator launch smoke loads home on iPhone 17 Pro and iPad Pro 13-inch; Home Screen/TestFlight review remains.</x:v>
       </x:c>
       <x:c r="L26" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46266</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
@@ -3225,7 +3225,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F54" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G54" s="21" t="str">
         <x:v>TECH-007</x:v>
@@ -3238,10 +3238,10 @@
         <x:v>APPLE-QA</x:v>
       </x:c>
       <x:c r="K54" s="21" t="str">
-        <x:v>Must pass on physical devices.</x:v>
+        <x:v>Clean-install and first-launch home-screen smoke passed on both simulators. Offline/online transitions and physical-device testing remain.</x:v>
       </x:c>
       <x:c r="L54" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46266</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
@@ -3409,7 +3409,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F59" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G59" s="21" t="str">
         <x:v>TECH-001</x:v>
@@ -3422,10 +3422,10 @@
         <x:v>APPLE-SUBMIT</x:v>
       </x:c>
       <x:c r="K59" s="21" t="str">
-        <x:v>Re-check Apple's upcoming requirements before future releases.</x:v>
+        <x:v>Xcode 26.6/iOS 26.5 simulator Debug builds succeeded on both devices. Release archive/signing remain; re-check Apple requirements before future releases.</x:v>
       </x:c>
       <x:c r="L59" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46266</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
@@ -3519,7 +3519,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7e5fbd02c5494b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a91e43efe7e405a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4139,7 +4139,7 @@
       </x:c>
       <x:c r="D36" s="27" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A36,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A36,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A36,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E36" s="21" t="str">
         <x:v>Update Task Register evidence here.</x:v>
@@ -4229,7 +4229,7 @@
       </x:c>
       <x:c r="D41" s="27" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A41,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A41,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A41,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E41" s="21" t="str">
         <x:v>Update Task Register evidence here.</x:v>
@@ -4264,7 +4264,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra276e95a6add4cef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racb3792ab3b54961"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4722,7 +4722,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36e11062d0484ca7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12c1291b0b2d4338"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5153,7 +5153,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red2016081e1e4d31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R886b85b1034e4cf7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Configure iOS device signing and app icon
</commit_message>
<xml_diff>
--- a/ios-app-readiness/iOS_App_Readiness_Tracker.xlsx
+++ b/ios-app-readiness/iOS_App_Readiness_Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9fb08bbe167643ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="2" r:id="Rf8180201b7964135"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checklist" sheetId="3" r:id="Rab250d69b01c4e0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Map" sheetId="4" r:id="R46bdab8948e14616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R12f1321f28574a3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3a578adf2f2945c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="2" r:id="Rbc968248c6d84965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checklist" sheetId="3" r:id="R2ca2adb5b7fd4f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Map" sheetId="4" r:id="R8dae4a494dad471d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R41a0404cd9234c95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -812,7 +812,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="37" t="str">
-        <x:v>Project-local source of truth for converting the Data Science Python Playground into a publishable iPhone/iPad app. Updated 2026-08-31.</x:v>
+        <x:v>Project-local source of truth for converting the Data Science Python Playground into a publishable iPhone/iPad app. Updated 2026-09-02.</x:v>
       </x:c>
       <x:c r="B2" s="37" t="str">
         <x:v>Project-local source of truth for converting the Data Science Python Playground into a publishable iPhone/iPad app. Updated 2026-08-31.</x:v>
@@ -870,12 +870,12 @@
       <x:c r="B5" s="47"/>
       <x:c r="C5" s="46" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"Done")</x:f>
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D5" s="47"/>
       <x:c r="E5" s="46" t="n">
         <x:f>A5-C5</x:f>
-        <x:v>38</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F5" s="47"/>
       <x:c r="G5" s="46" t="n">
@@ -912,7 +912,7 @@
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
       <x:c r="A8" s="69" t="str">
-        <x:v>Ship version 1 on Mac through the browser/GitHub Pages and use the shared Capacitor shell for iPhone/iPad. Sessions are intentionally temporary: backgrounding may preserve active work, but terminating the process returns to a fresh canvas. AdMob is the chosen future provider with banners only. Next gates are freeing space/installing full Xcode, Apple signing/device validation, publishing the legal URLs, and owner-created AdMob credentials.</x:v>
+        <x:v>Ship version 1 on Mac through the browser/GitHub Pages and use the shared Capacitor shell for iPhone/iPad. Sessions are intentionally temporary: backgrounding may preserve active work, but terminating the process returns to a fresh canvas. AdMob is the chosen future provider with banners only. Xcode 26.6 signing and iPad device launch validation now pass on a free Personal Team profile through 2026-09-09; next gates are full route/offline/device QA, publishing the legal URLs, owner-created AdMob credentials, and paid Apple Developer membership for App Store/TestFlight.</x:v>
       </x:c>
       <x:c r="B8" s="70" t="str">
         <x:v>Ship version 1 on Mac through the browser/GitHub Pages and use the shared Capacitor shell for iPhone/iPad. Sessions are intentionally temporary: backgrounding may preserve active work, but terminating the process returns to a fresh canvas. AdMob is the chosen future provider with banners only. Next gates are freeing space/installing full Xcode, Apple signing/device validation, publishing the legal URLs, and owner-created AdMob credentials.</x:v>
@@ -1047,14 +1047,15 @@
       <x:c r="D14" s="20" t="str">
         <x:v>Fresh canvas after termination</x:v>
       </x:c>
+      <x:c r="E14"/>
       <x:c r="F14" s="26" t="str">
-        <x:v>TECH-001</x:v>
+        <x:v>STORE-001</x:v>
       </x:c>
       <x:c r="G14" s="20" t="str">
-        <x:v>Free space + install Xcode</x:v>
+        <x:v>Enroll in paid Apple Developer Program</x:v>
       </x:c>
       <x:c r="H14" s="20" t="str">
-        <x:v>Needs explicit cache/release cleanup and App Store install confirmation</x:v>
+        <x:v>Needed for App Store/TestFlight; Personal Team expires 2026-09-09.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
@@ -1070,14 +1071,15 @@
       <x:c r="D15" s="21" t="str">
         <x:v>Browser-only Mac v1</x:v>
       </x:c>
+      <x:c r="E15"/>
       <x:c r="F15" s="27" t="str">
-        <x:v>TECH-002</x:v>
+        <x:v>QA-002</x:v>
       </x:c>
       <x:c r="G15" s="21" t="str">
-        <x:v>Register bundle identifier</x:v>
+        <x:v>Run iPhone/iPad workflow QA</x:v>
       </x:c>
       <x:c r="H15" s="21" t="str">
-        <x:v>Held until Apple Developer work resumes</x:v>
+        <x:v>Signed iPad launch passes; offline, Files, routes, and relaunch remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="26" customHeight="1">
@@ -1139,14 +1141,15 @@
       <x:c r="D18" s="21" t="str">
         <x:v>Automated route/runtime QA</x:v>
       </x:c>
+      <x:c r="E18"/>
       <x:c r="F18" s="27" t="str">
-        <x:v>QA-002</x:v>
+        <x:v>QA-004</x:v>
       </x:c>
       <x:c r="G18" s="21" t="str">
-        <x:v>Run iPhone/iPad device checks</x:v>
+        <x:v>Run physical-device performance QA</x:v>
       </x:c>
       <x:c r="H18" s="21" t="str">
-        <x:v>Requires full Xcode or physical devices</x:v>
+        <x:v>iPad is ready; profiling and large-runtime checks remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1267,7 +1270,7 @@
       </x:c>
       <x:c r="B26" s="26" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"Done")</x:f>
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
@@ -1276,7 +1279,7 @@
       </x:c>
       <x:c r="B27" s="27" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"In Progress")</x:f>
-        <x:v>18</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
@@ -1697,7 +1700,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F13" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G13" s="21" t="str">
         <x:v>DEC-001</x:v>
@@ -1706,16 +1709,16 @@
         <x:v>Developer</x:v>
       </x:c>
       <x:c r="I13" s="21" t="str">
-        <x:v>ios/; capacitor.config.json; package.json</x:v>
+        <x:v>ios/; capacitor.config.json; package.json; Xcode signing; paired iPad</x:v>
       </x:c>
       <x:c r="J13" s="21" t="str">
         <x:v>APPLE-SUBMIT</x:v>
       </x:c>
       <x:c r="K13" s="21" t="str">
-        <x:v>Capacitor 8 Xcode project created with approved bundle ID. Xcode 26.6 selected; first launch complete; iOS 26.5 simulator mounted; Swift packages resolved; unsigned Debug builds launch on iPhone 17 Pro/iPad Pro 13-inch. Signing/Developer enrollment remain.</x:v>
+        <x:v>Capacitor 8 Xcode project created with approved bundle ID. Xcode 26.6 installed; Apple Development certificate created for the free Personal Team; automatic signing enabled; Developer Mode enabled; Xcode-managed provisioning profile generated for the paired iPad (expires 2026-09-09). Signed Debug build installed and launched successfully on iPad Pro 13-inch M4 (iPadOS 26.6). Release archive/signing remains.</x:v>
       </x:c>
       <x:c r="L13" s="29" t="n">
-        <x:v>46266</x:v>
+        <x:v>46267</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -1735,7 +1738,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F14" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G14" s="21" t="str">
         <x:v>DEC-001</x:v>
@@ -1744,16 +1747,16 @@
         <x:v>Project owner</x:v>
       </x:c>
       <x:c r="I14" s="21" t="str">
-        <x:v>ios-app-architecture.md</x:v>
+        <x:v>ios-app-architecture.md; Xcode automatic signing; Personal Team</x:v>
       </x:c>
       <x:c r="J14" s="21" t="str">
         <x:v>APPLE-ACCOUNT</x:v>
       </x:c>
       <x:c r="K14" s="21" t="str">
-        <x:v>Approved ID: com.elijahang.datascienceplayground. Registration still requires Apple Developer account access.</x:v>
+        <x:v>Approved ID com.elijahang.datascienceplayground is registered through Xcode automatic signing under the free Personal Team; one physical iPad is registered. Paid Apple Developer Program enrollment remains required for App Store/TestFlight distribution and longer-lived profiles.</x:v>
       </x:c>
       <x:c r="L14" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46267</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -3233,15 +3236,17 @@
       <x:c r="H54" s="21" t="str">
         <x:v>QA</x:v>
       </x:c>
-      <x:c r="I54" s="21" t="str"/>
+      <x:c r="I54" s="21" t="str">
+        <x:v>iPad Pro 13-inch M4 (iPadOS 26.6); signed Debug build</x:v>
+      </x:c>
       <x:c r="J54" s="21" t="str">
         <x:v>APPLE-QA</x:v>
       </x:c>
       <x:c r="K54" s="21" t="str">
-        <x:v>Clean-install and first-launch home-screen smoke passed on both simulators. Offline/online transitions and physical-device testing remain.</x:v>
+        <x:v>Signed Debug build clean-install/first-launch smoke now passes on the physical iPad Pro 13-inch M4. Offline/online transitions, Files workflows, and relaunch behavior remain to be tested.</x:v>
       </x:c>
       <x:c r="L54" s="29" t="n">
-        <x:v>46266</x:v>
+        <x:v>46267</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
@@ -3417,15 +3422,17 @@
       <x:c r="H59" s="21" t="str">
         <x:v>Developer</x:v>
       </x:c>
-      <x:c r="I59" s="21" t="str"/>
+      <x:c r="I59" s="21" t="str">
+        <x:v>Xcode 26.6; iOS/iPadOS 26.5 SDK; iPad Pro 13-inch M4</x:v>
+      </x:c>
       <x:c r="J59" s="21" t="str">
         <x:v>APPLE-SUBMIT</x:v>
       </x:c>
       <x:c r="K59" s="21" t="str">
-        <x:v>Xcode 26.6/iOS 26.5 simulator Debug builds succeeded on both devices. Release archive/signing remain; re-check Apple requirements before future releases.</x:v>
+        <x:v>Xcode 26.6 and the iOS/iPadOS 26.5 SDK are installed. Signed Debug build is installed and running on iPad Pro 13-inch M4 (iPadOS 26.6) using the Personal Team profile. Release archive/signing remains incomplete.</x:v>
       </x:c>
       <x:c r="L59" s="29" t="n">
-        <x:v>46266</x:v>
+        <x:v>46267</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
@@ -3519,7 +3526,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a91e43efe7e405a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf841d03ae07e41c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3582,7 +3589,7 @@
       </x:c>
       <x:c r="D3" s="81" t="n">
         <x:f>COUNTIF(D7:D42,"Done")</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E3" s="82" t="str">
         <x:v>Derived from Task Register</x:v>
@@ -3617,10 +3624,10 @@
       </x:c>
       <x:c r="D7" s="26" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A7,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A7,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A7,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E7" s="20" t="str">
-        <x:v>ios/; capacitor.config.json; package.json</x:v>
+        <x:v>ios/; Xcode-managed signing; iPad Pro 13-inch M4 (iPadOS 26.6)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -4232,7 +4239,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E41" s="21" t="str">
-        <x:v>Update Task Register evidence here.</x:v>
+        <x:v>Xcode 26.6; iOS/iPadOS 26.5 SDK; signed Debug iPad build; release archive remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="30" customHeight="1">
@@ -4264,7 +4271,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racb3792ab3b54961"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bc8da6358ce4f27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4617,7 +4624,7 @@
         <x:v>TECH-001</x:v>
       </x:c>
       <x:c r="E21" s="21" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
@@ -4634,7 +4641,7 @@
         <x:v>TECH-001</x:v>
       </x:c>
       <x:c r="E22" s="21" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
@@ -4722,7 +4729,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12c1291b0b2d4338"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6034aecb5c4f4b6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5153,7 +5160,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R886b85b1034e4cf7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b9818c76d8e4ebc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: complete release license evidence
</commit_message>
<xml_diff>
--- a/ios-app-readiness/iOS_App_Readiness_Tracker.xlsx
+++ b/ios-app-readiness/iOS_App_Readiness_Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3a578adf2f2945c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="2" r:id="Rbc968248c6d84965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checklist" sheetId="3" r:id="R2ca2adb5b7fd4f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Map" sheetId="4" r:id="R8dae4a494dad471d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R41a0404cd9234c95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R46d254428c444c46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="2" r:id="Rd4462263ac754f96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checklist" sheetId="3" r:id="Rbc47ce709bb8469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Map" sheetId="4" r:id="R26a1146e96244f9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rb7f58172d46c4318"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -870,12 +870,12 @@
       <x:c r="B5" s="47"/>
       <x:c r="C5" s="46" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"Done")</x:f>
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D5" s="47"/>
       <x:c r="E5" s="46" t="n">
         <x:f>A5-C5</x:f>
-        <x:v>36</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F5" s="47"/>
       <x:c r="G5" s="46" t="n">
@@ -1270,7 +1270,7 @@
       </x:c>
       <x:c r="B26" s="26" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"Done")</x:f>
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
@@ -1279,7 +1279,7 @@
       </x:c>
       <x:c r="B27" s="27" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"In Progress")</x:f>
-        <x:v>16</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
@@ -1835,7 +1835,7 @@
         <x:v>46265</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="42" customHeight="1">
+    <x:row r="17" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A17" s="25" t="str">
         <x:v>TECH-005</x:v>
       </x:c>
@@ -1852,7 +1852,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F17" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G17" s="21" t="str">
         <x:v>TECH-004</x:v>
@@ -1861,16 +1861,16 @@
         <x:v>Developer</x:v>
       </x:c>
       <x:c r="I17" s="21" t="str">
-        <x:v>scripts/vendor-pyodide.mjs; vendor/pyodide/runtime-manifest.json</x:v>
+        <x:v>scripts/vendor-pyodide.mjs; vendor/pyodide/runtime-manifest.json; iPad Pro 13-inch M4 (iPadOS 26.6)</x:v>
       </x:c>
       <x:c r="J17" s="21" t="str">
         <x:v>PROJECT</x:v>
       </x:c>
       <x:c r="K17" s="21" t="str">
-        <x:v>Pinned 146 MB runtime/package closure built and browser-smoke tested. npm ci, npm run ios:sync, and npm run check pass. Clean-install simulator launch reached home; offline/runtime recovery still needs validation.</x:v>
+        <x:v>Pinned 146 MB runtime/package closure built and browser-smoke tested. npm ci, npm run ios:sync, and npm run check pass. Clean-install launch and the owner's 2026-09-04 offline cold-launch test (bundled dataset selection and cell execution with Wi-Fi disabled) pass on the physical iPad Pro 13-inch M4.</x:v>
       </x:c>
       <x:c r="L17" s="29" t="n">
-        <x:v>46266</x:v>
+        <x:v>46269</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
@@ -2023,7 +2023,7 @@
         <x:v>46265</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="42" customHeight="1">
+    <x:row r="22" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A22" s="25" t="str">
         <x:v>TECH-010</x:v>
       </x:c>
@@ -2049,19 +2049,19 @@
         <x:v>Developer</x:v>
       </x:c>
       <x:c r="I22" s="21" t="str">
-        <x:v>app/app-platform.js; playground.html; ml-app.js</x:v>
+        <x:v>app/app-platform.js; playground.html; ml-app.js; iPad Pro 13-inch M4 (iPadOS 26.6)</x:v>
       </x:c>
       <x:c r="J22" s="21" t="str">
         <x:v>CAPACITOR</x:v>
       </x:c>
       <x:c r="K22" s="21" t="str">
-        <x:v>CSV/chart exports now write a temporary native file and invoke Share Sheet. Physical Files/Share testing remains.</x:v>
+        <x:v>CSV/chart exports now write a temporary native file and invoke Share Sheet. The owner confirmed the Share Sheet opens on the physical iPad on 2026-09-04; Save to Files/result validation remains.</x:v>
       </x:c>
       <x:c r="L22" s="29" t="n">
-        <x:v>46265</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="42" customHeight="1">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A23" s="25" t="str">
         <x:v>TECH-011</x:v>
       </x:c>
@@ -2078,7 +2078,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F23" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G23" s="21" t="str">
         <x:v>TECH-001</x:v>
@@ -2087,16 +2087,16 @@
         <x:v>Developer</x:v>
       </x:c>
       <x:c r="I23" s="21" t="str">
-        <x:v>app/app-platform.js</x:v>
+        <x:v>app/app-platform.js; iPad Pro 13-inch M4 (iPadOS 26.6)</x:v>
       </x:c>
       <x:c r="J23" s="21" t="str">
         <x:v>APPLE-QA</x:v>
       </x:c>
       <x:c r="K23" s="21" t="str">
-        <x:v>External HTTP(S) links are routed through Capacitor Browser; native presentation/dismissal still needs device validation.</x:v>
+        <x:v>External HTTPS links are routed through Capacitor Browser; the owner confirmed the in-app browser opens and dismisses correctly on the physical iPad on 2026-09-04.</x:v>
       </x:c>
       <x:c r="L23" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46269</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
@@ -2213,7 +2213,7 @@
         <x:v>46266</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="42" customHeight="1">
+    <x:row r="27" ht="66" hidden="0" customHeight="1">
       <x:c r="A27" s="25" t="str">
         <x:v>UX-002</x:v>
       </x:c>
@@ -2239,16 +2239,16 @@
         <x:v>Developer</x:v>
       </x:c>
       <x:c r="I27" s="21" t="str">
-        <x:v>home.css; playground.html; ml.html</x:v>
+        <x:v>home.css; playground.html; ml.html; iPad Pro 13-inch M4 (iPadOS 26.6)</x:v>
       </x:c>
       <x:c r="J27" s="21" t="str">
         <x:v>APPLE-QA</x:v>
       </x:c>
       <x:c r="K27" s="21" t="str">
-        <x:v>Responsive and safe-area work is implemented and desktop mobile-viewport checks pass. iOS keyboard, touch, rotation, and panels need devices.</x:v>
+        <x:v>Responsive and safe-area work is implemented and desktop mobile-viewport checks pass. The owner confirmed portrait/landscape rotation on the physical iPad on 2026-09-04. Independent cell/output scrolling changes are pending native-app sync and revalidation.</x:v>
       </x:c>
       <x:c r="L27" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46269</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
@@ -3211,7 +3211,7 @@
         <x:v>46265</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="42" customHeight="1">
+    <x:row r="54" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A54" s="25" t="str">
         <x:v>QA-002</x:v>
       </x:c>
@@ -3237,19 +3237,19 @@
         <x:v>QA</x:v>
       </x:c>
       <x:c r="I54" s="21" t="str">
-        <x:v>iPad Pro 13-inch M4 (iPadOS 26.6); signed Debug build</x:v>
+        <x:v>iPad Pro 13-inch M4 (iPadOS 26.6); signed Debug build; physical offline cold-launch check</x:v>
       </x:c>
       <x:c r="J54" s="21" t="str">
         <x:v>APPLE-QA</x:v>
       </x:c>
       <x:c r="K54" s="21" t="str">
-        <x:v>Signed Debug build clean-install/first-launch smoke now passes on the physical iPad Pro 13-inch M4. Offline/online transitions, Files workflows, and relaunch behavior remain to be tested.</x:v>
+        <x:v>Signed Debug build clean-install/first-launch smoke and offline runtime execution now pass on the physical iPad Pro 13-inch M4. The owner confirmed Wi-Fi-disabled cold relaunch, bundled dataset selection, and one-cell execution on 2026-09-04; full online/offline transition and retry matrix remains.</x:v>
       </x:c>
       <x:c r="L54" s="29" t="n">
-        <x:v>46267</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55" ht="42" customHeight="1">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A55" s="25" t="str">
         <x:v>QA-003</x:v>
       </x:c>
@@ -3275,16 +3275,16 @@
         <x:v>QA</x:v>
       </x:c>
       <x:c r="I55" s="21" t="str">
-        <x:v>tests/; .github/workflows/ml-route-audit.yml</x:v>
+        <x:v>tests/; .github/workflows/ml-route-audit.yml; iPad Pro 13-inch M4 (iPadOS 26.6) bundled dataset check</x:v>
       </x:c>
       <x:c r="J55" s="21" t="str">
         <x:v>PROJECT</x:v>
       </x:c>
       <x:c r="K55" s="21" t="str">
-        <x:v>Fast 254-route checks and bundled-runtime browser smoke pass. Representative iOS device journeys remain.</x:v>
+        <x:v>Fast 254-route checks and bundled-runtime browser smoke pass. The owner confirmed bundled dataset selection and cell execution on the physical iPad on 2026-09-04; full representative route/dataset matrix remains.</x:v>
       </x:c>
       <x:c r="L55" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46269</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
@@ -3323,7 +3323,7 @@
         <x:v>46265</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="42" customHeight="1">
+    <x:row r="57" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A57" s="25" t="str">
         <x:v>QA-005</x:v>
       </x:c>
@@ -3340,7 +3340,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F57" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G57" s="21" t="str">
         <x:v>TECH-012</x:v>
@@ -3349,16 +3349,16 @@
         <x:v>QA</x:v>
       </x:c>
       <x:c r="I57" s="21" t="str">
-        <x:v>app/app-platform.js; ios-app-architecture.md</x:v>
+        <x:v>app/app-platform.js; ios-app-architecture.md; physical iPad background/relaunch checks</x:v>
       </x:c>
       <x:c r="J57" s="21" t="str">
         <x:v>APPLE-QA</x:v>
       </x:c>
       <x:c r="K57" s="21" t="str">
-        <x:v>No disk persistence is intentional and documented. Continuity while backgrounded and reset after process termination still need simulator/device validation.</x:v>
+        <x:v>No disk persistence is intentional and documented. The owner confirmed active work remains after backgrounding and returns to a fresh canvas after swipe-kill/reopen on the physical iPad on 2026-09-04.</x:v>
       </x:c>
       <x:c r="L57" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46269</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
@@ -3526,7 +3526,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf841d03ae07e41c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a23da99ccd6439e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3589,7 +3589,7 @@
       </x:c>
       <x:c r="D3" s="81" t="n">
         <x:f>COUNTIF(D7:D42,"Done")</x:f>
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E3" s="82" t="str">
         <x:v>Derived from Task Register</x:v>
@@ -3648,7 +3648,7 @@
         <x:v>scripts/build-web.mjs; capacitor.config.json; ios/App/App/public/</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="30" customHeight="1">
+    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A9" s="25" t="str">
         <x:v>TECH-005</x:v>
       </x:c>
@@ -3660,10 +3660,10 @@
       </x:c>
       <x:c r="D9" s="27" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A9,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A9,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A9,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E9" s="21" t="str">
-        <x:v>scripts/vendor-pyodide.mjs; vendor/pyodide/runtime-manifest.json</x:v>
+        <x:v>scripts/vendor-pyodide.mjs; vendor/pyodide/runtime-manifest.json; physical iPad offline cold-launch check</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
@@ -3720,7 +3720,7 @@
         <x:v>playground.html; ios/App/App/Info.plist</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="30" customHeight="1">
+    <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A13" s="25" t="str">
         <x:v>TECH-010</x:v>
       </x:c>
@@ -3735,7 +3735,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E13" s="21" t="str">
-        <x:v>app/app-platform.js; playground.html; ml-app.js</x:v>
+        <x:v>app/app-platform.js; playground.html; ml-app.js; physical iPad Share Sheet check (Save to Files/result validation remains)</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
@@ -3756,7 +3756,7 @@
         <x:v>assets/icons/; ios/App/App/Assets.xcassets; ios/App/App/Info.plist</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="30" customHeight="1">
+    <x:row r="15" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A15" s="25" t="str">
         <x:v>UX-002</x:v>
       </x:c>
@@ -3771,7 +3771,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E15" s="21" t="str">
-        <x:v>home.css; playground.html; ml.html</x:v>
+        <x:v>home.css; playground.html; ml.html; physical iPad rotation check; independent cell/output scrolling update pending native revalidation</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
@@ -4134,7 +4134,7 @@
         <x:v>Update Task Register evidence here.</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="30" customHeight="1">
+    <x:row r="36" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A36" s="25" t="str">
         <x:v>QA-002</x:v>
       </x:c>
@@ -4149,10 +4149,10 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E36" s="21" t="str">
-        <x:v>Update Task Register evidence here.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="30" customHeight="1">
+        <x:v>Physical iPad clean-install/first-launch smoke; Wi-Fi-disabled cold relaunch, bundled dataset, and one-cell execution confirmed; online/offline transition and retry matrix remains</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A37" s="25" t="str">
         <x:v>QA-003</x:v>
       </x:c>
@@ -4167,7 +4167,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E37" s="21" t="str">
-        <x:v>tests/; .github/workflows/ml-route-audit.yml</x:v>
+        <x:v>tests/; .github/workflows/ml-route-audit.yml; physical iPad bundled dataset check; full representative route/dataset matrix remains</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="30" customHeight="1">
@@ -4188,7 +4188,7 @@
         <x:v>Update Task Register evidence here.</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="30" customHeight="1">
+    <x:row r="39" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A39" s="25" t="str">
         <x:v>QA-005</x:v>
       </x:c>
@@ -4200,10 +4200,10 @@
       </x:c>
       <x:c r="D39" s="27" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A39,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A39,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A39,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E39" s="21" t="str">
-        <x:v>app/app-platform.js; ios-app-architecture.md</x:v>
+        <x:v>app/app-platform.js; ios-app-architecture.md; physical iPad background/relaunch checks confirmed</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="30" customHeight="1">
@@ -4271,7 +4271,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bc8da6358ce4f27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R701c0d569e474533"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4729,7 +4729,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6034aecb5c4f4b6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R287892895aa14c3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5160,7 +5160,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b9818c76d8e4ebc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00e9075135c54f18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record completed release QA gates
</commit_message>
<xml_diff>
--- a/ios-app-readiness/iOS_App_Readiness_Tracker.xlsx
+++ b/ios-app-readiness/iOS_App_Readiness_Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R46d254428c444c46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="2" r:id="Rd4462263ac754f96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checklist" sheetId="3" r:id="Rbc47ce709bb8469e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Map" sheetId="4" r:id="R26a1146e96244f9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rb7f58172d46c4318"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R54b9c181022f4b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="2" r:id="Rb5a72c597d5b4a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checklist" sheetId="3" r:id="R098bd5605dc74491"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Map" sheetId="4" r:id="R1e43e71313b54657"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R0c2b56588f1d4328"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -812,7 +812,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="37" t="str">
-        <x:v>Project-local source of truth for converting the Data Science Python Playground into a publishable iPhone/iPad app. Updated 2026-09-02.</x:v>
+        <x:v>Project-local source of truth for converting the Data Science Python Playground into a publishable iPhone/iPad app. Updated 2026-09-04.</x:v>
       </x:c>
       <x:c r="B2" s="37" t="str">
         <x:v>Project-local source of truth for converting the Data Science Python Playground into a publishable iPhone/iPad app. Updated 2026-08-31.</x:v>
@@ -870,12 +870,12 @@
       <x:c r="B5" s="47"/>
       <x:c r="C5" s="46" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"Done")</x:f>
-        <x:v>24</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D5" s="47"/>
       <x:c r="E5" s="46" t="n">
         <x:f>A5-C5</x:f>
-        <x:v>33</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F5" s="47"/>
       <x:c r="G5" s="46" t="n">
@@ -1110,10 +1110,10 @@
         <x:v>PRIV-005</x:v>
       </x:c>
       <x:c r="B17" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="C17" s="21" t="str">
-        <x:v>acknowledgements.html; licenses/</x:v>
+        <x:v>acknowledgements.html; assets/licenses/manifest.json</x:v>
       </x:c>
       <x:c r="D17" s="21" t="str">
         <x:v>Rights evidence and notices</x:v>
@@ -1133,10 +1133,10 @@
         <x:v>QA-003</x:v>
       </x:c>
       <x:c r="B18" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="C18" s="21" t="str">
-        <x:v>tests/; CI workflow</x:v>
+        <x:v>tests/; .github/workflows/ml-route-audit.yml; main b13c314</x:v>
       </x:c>
       <x:c r="D18" s="21" t="str">
         <x:v>Automated route/runtime QA</x:v>
@@ -1270,7 +1270,7 @@
       </x:c>
       <x:c r="B26" s="26" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"Done")</x:f>
-        <x:v>24</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
@@ -1279,7 +1279,7 @@
       </x:c>
       <x:c r="B27" s="27" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"In Progress")</x:f>
-        <x:v>13</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
@@ -1297,7 +1297,7 @@
       </x:c>
       <x:c r="B29" s="27" t="n">
         <x:f>COUNTIF('Task Register'!$F$5:$F$61,"Not Started")</x:f>
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2437,7 +2437,7 @@
         <x:v>46265</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="42" customHeight="1">
+    <x:row r="33" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A33" s="25" t="str">
         <x:v>PRIV-003</x:v>
       </x:c>
@@ -2454,7 +2454,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F33" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G33" s="21" t="str">
         <x:v>PRIV-002</x:v>
@@ -2463,16 +2463,16 @@
         <x:v>Developer</x:v>
       </x:c>
       <x:c r="I33" s="21" t="str">
-        <x:v>ios/App/App/PrivacyInfo.xcprivacy</x:v>
+        <x:v>ios/App/App/PrivacyInfo.xcprivacy; ios/App/App/Info.plist; privacy manifest/plist lint; Release archive parity audit</x:v>
       </x:c>
       <x:c r="J33" s="21" t="str">
         <x:v>APPLE-MANIFEST</x:v>
       </x:c>
       <x:c r="K33" s="21" t="str">
-        <x:v>Initial required-reason manifest is valid XML and included in the Xcode resources. Final archive/SDK manifest validation remains.</x:v>
+        <x:v>Required-reason privacy manifest is valid XML and included in the Xcode resources. Final privacy-manifest/plist lint and Release archive parity passed on 2026-09-04.</x:v>
       </x:c>
       <x:c r="L33" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46269</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
@@ -2513,7 +2513,7 @@
         <x:v>46265</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="42" customHeight="1">
+    <x:row r="35" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A35" s="25" t="str">
         <x:v>PRIV-005</x:v>
       </x:c>
@@ -2530,7 +2530,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F35" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G35" s="21" t="str">
         <x:v>TECH-006</x:v>
@@ -2539,16 +2539,16 @@
         <x:v>Project owner</x:v>
       </x:c>
       <x:c r="I35" s="21" t="str">
-        <x:v>acknowledgements.html; assets/licenses/manifest.json; third-party-rights-and-licenses.md</x:v>
+        <x:v>acknowledgements.html; assets/licenses/manifest.json; third-party-rights-and-licenses.md; Release archive parity audit</x:v>
       </x:c>
       <x:c r="J35" s="21" t="str">
         <x:v>APPLE-RIGHTS</x:v>
       </x:c>
       <x:c r="K35" s="21" t="str">
-        <x:v>Public credits and 52 exact notices cover datasets, fonts, Capacitor, and Python wheels. Final Palmer publication-policy and release-archive reconciliation remain.</x:v>
+        <x:v>Public credits and 55 exact notices, including synapse, capacitor-swift-pm, and ion-ios-filesystem, cover the shipped datasets, fonts, Capacitor, and Python wheels. Acknowledgements and the Palmer 333-row complete-case subset match the final Release archive; no license-specific blocker remains.</x:v>
       </x:c>
       <x:c r="L35" s="29" t="n">
-        <x:v>46265</x:v>
+        <x:v>46269</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
@@ -3249,7 +3249,7 @@
         <x:v>46269</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="55" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A55" s="25" t="str">
         <x:v>QA-003</x:v>
       </x:c>
@@ -3266,7 +3266,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F55" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G55" s="21" t="str">
         <x:v>TECH-008</x:v>
@@ -3275,13 +3275,13 @@
         <x:v>QA</x:v>
       </x:c>
       <x:c r="I55" s="21" t="str">
-        <x:v>tests/; .github/workflows/ml-route-audit.yml; iPad Pro 13-inch M4 (iPadOS 26.6) bundled dataset check</x:v>
+        <x:v>tests/; .github/workflows/ml-route-audit.yml; main b13c314 254-route runtime audit; iPhone 17e iOS 26.5 simulator; local browser/Pyodide smoke; physical iPad bundled dataset check</x:v>
       </x:c>
       <x:c r="J55" s="21" t="str">
         <x:v>PROJECT</x:v>
       </x:c>
       <x:c r="K55" s="21" t="str">
-        <x:v>Fast 254-route checks and bundled-runtime browser smoke pass. The owner confirmed bundled dataset selection and cell execution on the physical iPad on 2026-09-04; full representative route/dataset matrix remains.</x:v>
+        <x:v>The full 254-route runtime audit on main b13c314 passes, alongside local browser/Pyodide smoke and iPhone 17e iOS 26.5 simulator build/install/launch. The owner also confirmed bundled dataset selection and cell execution on the physical iPad on 2026-09-04.</x:v>
       </x:c>
       <x:c r="L55" s="29" t="n">
         <x:v>46269</x:v>
@@ -3361,7 +3361,7 @@
         <x:v>46269</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="42" customHeight="1">
+    <x:row r="58" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A58" s="25" t="str">
         <x:v>QA-006</x:v>
       </x:c>
@@ -3378,7 +3378,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F58" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G58" s="21" t="str">
         <x:v>PRIV-003</x:v>
@@ -3386,18 +3386,20 @@
       <x:c r="H58" s="21" t="str">
         <x:v>QA</x:v>
       </x:c>
-      <x:c r="I58" s="21" t="str"/>
+      <x:c r="I58" s="21" t="str">
+        <x:v>npm check; tests/; iPhone 17e iOS 26.5 simulator; local browser/Pyodide smoke; ios/App/App/PrivacyInfo.xcprivacy; ios/App/App/Info.plist; npm production audit</x:v>
+      </x:c>
       <x:c r="J58" s="21" t="str">
         <x:v>APPLE-PRIVACY</x:v>
       </x:c>
       <x:c r="K58" s="21" t="str">
-        <x:v>Complete immediately before archive.</x:v>
+        <x:v>Final privacy, accessibility, and security regression passes: npm check, the 254-route runtime audit, simulator build/install/launch, local browser/Pyodide smoke, privacy manifest/plist lint, and npm production audit with 0 vulnerabilities. No sensitive permissions, cross-app tracking, persistence, or secrets were found.</x:v>
       </x:c>
       <x:c r="L58" s="29" t="n">
-        <x:v>46265</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="42" customHeight="1">
+        <x:v>46269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A59" s="25" t="str">
         <x:v>REL-001</x:v>
       </x:c>
@@ -3414,7 +3416,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F59" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G59" s="21" t="str">
         <x:v>TECH-001</x:v>
@@ -3423,16 +3425,16 @@
         <x:v>Developer</x:v>
       </x:c>
       <x:c r="I59" s="21" t="str">
-        <x:v>Xcode 26.6; iOS/iPadOS 26.5 SDK; iPad Pro 13-inch M4</x:v>
+        <x:v>Xcode 26.6; iOS/iPadOS 26.5 SDK; iPad Pro 13-inch M4; final Release archive parity audit</x:v>
       </x:c>
       <x:c r="J59" s="21" t="str">
         <x:v>APPLE-SUBMIT</x:v>
       </x:c>
       <x:c r="K59" s="21" t="str">
-        <x:v>Xcode 26.6 and the iOS/iPadOS 26.5 SDK are installed. Signed Debug build is installed and running on iPad Pro 13-inch M4 (iPadOS 26.6) using the Personal Team profile. Release archive/signing remains incomplete.</x:v>
+        <x:v>Xcode 26.6 and the iOS/iPadOS 26.5 SDK are installed. Final Release archive parity passed on 2026-09-04, including the generated runtime, acknowledgements, dataset, license bundle, and native package payloads.</x:v>
       </x:c>
       <x:c r="L59" s="29" t="n">
-        <x:v>46267</x:v>
+        <x:v>46269</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
@@ -3526,7 +3528,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a23da99ccd6439e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cf0c05dd96c4d8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3589,7 +3591,7 @@
       </x:c>
       <x:c r="D3" s="81" t="n">
         <x:f>COUNTIF(D7:D42,"Done")</x:f>
-        <x:v>9</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E3" s="82" t="str">
         <x:v>Derived from Task Register</x:v>
@@ -3846,7 +3848,7 @@
         <x:v>data-flow-audit.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="30" customHeight="1">
+    <x:row r="20" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A20" s="25" t="str">
         <x:v>PRIV-003</x:v>
       </x:c>
@@ -3858,13 +3860,13 @@
       </x:c>
       <x:c r="D20" s="27" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A20,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A20,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A20,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E20" s="21" t="str">
-        <x:v>ios/App/App/PrivacyInfo.xcprivacy</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="30" customHeight="1">
+        <x:v>ios/App/App/PrivacyInfo.xcprivacy; ios/App/App/Info.plist; privacy manifest/plist lint; Release archive parity passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="66" hidden="0" customHeight="1">
       <x:c r="A21" s="25" t="str">
         <x:v>PRIV-005</x:v>
       </x:c>
@@ -3876,10 +3878,10 @@
       </x:c>
       <x:c r="D21" s="27" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A21,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A21,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A21,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E21" s="21" t="str">
-        <x:v>acknowledgements.html; assets/licenses/manifest.json; third-party-rights-and-licenses.md</x:v>
+        <x:v>acknowledgements.html; assets/licenses/manifest.json; third-party-rights-and-licenses.md; 55-notice archive parity; Palmer 333-row complete-case parity; no license-specific blocker</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
@@ -4152,7 +4154,7 @@
         <x:v>Physical iPad clean-install/first-launch smoke; Wi-Fi-disabled cold relaunch, bundled dataset, and one-cell execution confirmed; online/offline transition and retry matrix remains</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="37" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A37" s="25" t="str">
         <x:v>QA-003</x:v>
       </x:c>
@@ -4164,10 +4166,10 @@
       </x:c>
       <x:c r="D37" s="27" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A37,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A37,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A37,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E37" s="21" t="str">
-        <x:v>tests/; .github/workflows/ml-route-audit.yml; physical iPad bundled dataset check; full representative route/dataset matrix remains</x:v>
+        <x:v>tests/; .github/workflows/ml-route-audit.yml; main b13c314 254-route runtime audit; iPhone 17e simulator; local browser/Pyodide smoke; physical iPad bundled dataset check</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="30" customHeight="1">
@@ -4206,7 +4208,7 @@
         <x:v>app/app-platform.js; ios-app-architecture.md; physical iPad background/relaunch checks confirmed</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="30" customHeight="1">
+    <x:row r="40" ht="66" hidden="0" customHeight="1">
       <x:c r="A40" s="25" t="str">
         <x:v>QA-006</x:v>
       </x:c>
@@ -4218,13 +4220,13 @@
       </x:c>
       <x:c r="D40" s="27" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A40,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A40,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A40,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>Not Started</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E40" s="21" t="str">
-        <x:v>Update Task Register evidence here.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="30" customHeight="1">
+        <x:v>npm check; 254-route runtime audit; iPhone 17e simulator; local browser/Pyodide smoke; privacy manifest/plist lint; npm production audit (0 vulnerabilities); no sensitive permissions/tracking/persistence/secrets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A41" s="25" t="str">
         <x:v>REL-001</x:v>
       </x:c>
@@ -4236,10 +4238,10 @@
       </x:c>
       <x:c r="D41" s="27" t="str">
         <x:f>IF(COUNTIFS('Task Register'!$A$5:$A$61,A41,'Task Register'!$F$5:$F$61,"Done")&gt;0,"Done",IF(COUNTIFS('Task Register'!$A$5:$A$61,A41,'Task Register'!$F$5:$F$61,"In Progress")&gt;0,"In Progress",IF(COUNTIFS('Task Register'!$A$5:$A$61,A41,'Task Register'!$F$5:$F$61,"Needs User Info")&gt;0,"Needs User Info","Not Started")))</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E41" s="21" t="str">
-        <x:v>Xcode 26.6; iOS/iPadOS 26.5 SDK; signed Debug iPad build; release archive remains.</x:v>
+        <x:v>Xcode 26.6; iOS/iPadOS 26.5 SDK; final Release archive parity passed</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="30" customHeight="1">
@@ -4271,7 +4273,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R701c0d569e474533"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2e4b9fb58a542e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4729,7 +4731,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R287892895aa14c3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8e4c27fdbf5469b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5160,7 +5162,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00e9075135c54f18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e899005b0874551"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>